<commit_message>
sync: align employee localisations with online dependants and keep both stores in sync
Pull latest dependants sites (Lubumbashi, MOANDA, Kisangani), update employee localisations, bidirectional sync on future edits, and expand dependants export RESUME sites.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Excel/templates/dependants/DEPENDANTS_EXPORT_TEMPLATE.xlsx
+++ b/Excel/templates/dependants/DEPENDANTS_EXPORT_TEMPLATE.xlsx
@@ -2442,6 +2442,15 @@
   </si>
   <si>
     <t>NaN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lubumbashi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOANDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kisangani</t>
   </si>
 </sst>
 </file>
@@ -5923,18 +5932,10 @@
       <c r="A28" t="s" s="60">
         <v>0</v>
       </c>
-      <c r="B28" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Zamba",DEPENDANTS!$D$3:$D$725,"*Employ*")</f>
-      </c>
-      <c r="C28" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Zamba",DEPENDANTS!$D$3:$D$725,"*Conjoint*")</f>
-      </c>
-      <c r="D28" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Zamba",DEPENDANTS!$D$3:$D$725,"Enfant")</f>
-      </c>
-      <c r="E28" s="69">
-        <f>SUM(B28:D28)</f>
-      </c>
+      <c r="B28" s="61"/>
+      <c r="C28" s="61"/>
+      <c r="D28" s="61"/>
+      <c r="E28" s="69"/>
       <c r="F28" s="70"/>
       <c r="G28" s="44"/>
       <c r="H28" s="44"/>
@@ -5957,18 +5958,10 @@
       <c r="A29" t="s" s="60">
         <v>177</v>
       </c>
-      <c r="B29" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Kinshasa",DEPENDANTS!$D$3:$D$725,"*Employ*")</f>
-      </c>
-      <c r="C29" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Kinshasa",DEPENDANTS!$D$3:$D$725,"*Conjoint*")</f>
-      </c>
-      <c r="D29" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Kinshasa",DEPENDANTS!$D$3:$D$725,"Enfant")</f>
-      </c>
-      <c r="E29" s="69">
-        <f>SUM(B29:D29)</f>
-      </c>
+      <c r="B29" s="61"/>
+      <c r="C29" s="61"/>
+      <c r="D29" s="61"/>
+      <c r="E29" s="69"/>
       <c r="F29" s="70"/>
       <c r="G29" s="44"/>
       <c r="H29" s="44"/>
@@ -5991,18 +5984,10 @@
       <c r="A30" t="s" s="60">
         <v>747</v>
       </c>
-      <c r="B30" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Lubudi",DEPENDANTS!$D$3:$D$725,"*Employ*")</f>
-      </c>
-      <c r="C30" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Lubudi",DEPENDANTS!$D$3:$D$725,"*Conjoint*")</f>
-      </c>
-      <c r="D30" s="61">
-        <f>COUNTIFS(DEPENDANTS!$G$3:$G$725,"Lubudi",DEPENDANTS!$D$3:$D$725,"Enfant")</f>
-      </c>
-      <c r="E30" s="69">
-        <f>SUM(B30:D30)</f>
-      </c>
+      <c r="B30" s="61"/>
+      <c r="C30" s="61"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="69"/>
       <c r="F30" s="70"/>
       <c r="G30" s="44"/>
       <c r="H30" s="44"/>
@@ -6023,20 +6008,12 @@
     </row>
     <row r="31" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s" s="64">
-        <v>753</v>
-      </c>
-      <c r="B31" s="65">
-        <f>SUM(B28:B30)</f>
-      </c>
-      <c r="C31" s="65">
-        <f>SUM(C28:C30)</f>
-      </c>
-      <c r="D31" s="65">
-        <f>SUM(D28:D30)</f>
-      </c>
-      <c r="E31" s="71">
-        <f>SUM(E28:E30)</f>
-      </c>
+        <v>800</v>
+      </c>
+      <c r="B31" s="65"/>
+      <c r="C31" s="65"/>
+      <c r="D31" s="65"/>
+      <c r="E31" s="71"/>
       <c r="F31" s="72"/>
       <c r="G31" s="44"/>
       <c r="H31" s="44"/>
@@ -6056,7 +6033,9 @@
       <c r="V31" s="33"/>
     </row>
     <row r="32" spans="1:22" ht="13" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2"/>
+      <c r="A32" t="s" s="2">
+        <v>801</v>
+      </c>
       <c r="B32" s="29"/>
       <c r="C32" s="29"/>
       <c r="D32" s="29"/>
@@ -6081,7 +6060,7 @@
     </row>
     <row r="33" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s" s="67">
-        <v>754</v>
+        <v>802</v>
       </c>
       <c r="B33" s="54"/>
       <c r="C33" s="54"/>
@@ -6107,17 +6086,11 @@
     </row>
     <row r="34" spans="1:6" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A34" t="s" s="57">
-        <v>207</v>
-      </c>
-      <c r="B34" t="s" s="58">
-        <v>755</v>
-      </c>
-      <c r="C34" t="s" s="58">
-        <v>756</v>
-      </c>
-      <c r="D34" t="s" s="58">
-        <v>4</v>
-      </c>
+        <v>753</v>
+      </c>
+      <c r="B34" s="58"/>
+      <c r="C34" s="58"/>
+      <c r="D34" s="58"/>
       <c r="E34" s="59"/>
       <c r="F34" s="44"/>
       <c r="G34" s="44"/>
@@ -6138,18 +6111,10 @@
       <c r="V34" s="33"/>
     </row>
     <row r="35" spans="1:6" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s" s="60">
-        <v>0</v>
-      </c>
-      <c r="B35" s="61">
-        <f ca="1">COUNTIFS(DEPENDANTS!$G$3:$G$725,"Zamba",DEPENDANTS!$I$3:$I$725,"&lt;=17")</f>
-      </c>
-      <c r="C35" s="61">
-        <f ca="1">COUNTIF(DEPENDANTS!$G$3:$G$725,"Zamba")-B35</f>
-      </c>
-      <c r="D35" s="62">
-        <f ca="1">SUM(B35:C35)</f>
-      </c>
+      <c r="A35" s="60"/>
+      <c r="B35" s="61"/>
+      <c r="C35" s="61"/>
+      <c r="D35" s="62"/>
       <c r="E35" s="63"/>
       <c r="F35" s="44"/>
       <c r="G35" s="44"/>
@@ -6171,17 +6136,11 @@
     </row>
     <row r="36" spans="1:6" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A36" t="s" s="60">
-        <v>177</v>
-      </c>
-      <c r="B36" s="61">
-        <f ca="1">COUNTIFS(DEPENDANTS!$G$3:$G$725,"Kinshasa",DEPENDANTS!$I$3:$I$725,"&lt;=17")</f>
-      </c>
-      <c r="C36" s="61">
-        <f ca="1">COUNTIF(DEPENDANTS!$G$3:$G$725,"Kinshasa")-B36</f>
-      </c>
-      <c r="D36" s="62">
-        <f ca="1">SUM(B36:C36)</f>
-      </c>
+        <v>754</v>
+      </c>
+      <c r="B36" s="61"/>
+      <c r="C36" s="61"/>
+      <c r="D36" s="62"/>
       <c r="E36" s="63"/>
       <c r="F36" s="44"/>
       <c r="G36" s="44"/>
@@ -6203,16 +6162,16 @@
     </row>
     <row r="37" spans="1:6" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A37" t="s" s="60">
-        <v>747</v>
-      </c>
-      <c r="B37" s="61">
-        <f ca="1">COUNTIFS(DEPENDANTS!$G$3:$G$725,"Lubudi",DEPENDANTS!$I$3:$I$725,"&lt;=17")</f>
-      </c>
-      <c r="C37" s="61">
-        <f ca="1">COUNTIF(DEPENDANTS!$G$3:$G$725,"Lubudi")-B37</f>
-      </c>
-      <c r="D37" s="62">
-        <f ca="1">SUM(B37:C37)</f>
+        <v>207</v>
+      </c>
+      <c r="B37" t="s" s="61">
+        <v>755</v>
+      </c>
+      <c r="C37" t="s" s="61">
+        <v>756</v>
+      </c>
+      <c r="D37" t="s" s="62">
+        <v>4</v>
       </c>
       <c r="E37" s="63"/>
       <c r="F37" s="44"/>
@@ -6235,17 +6194,11 @@
     </row>
     <row r="38" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s" s="64">
-        <v>753</v>
-      </c>
-      <c r="B38" s="65">
-        <f ca="1">SUM(B35:B37)</f>
-      </c>
-      <c r="C38" s="65">
-        <f ca="1">SUM(C35:C37)</f>
-      </c>
-      <c r="D38" s="65">
-        <f ca="1">SUM(D35:D37)</f>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B38" s="65"/>
+      <c r="C38" s="65"/>
+      <c r="D38" s="65"/>
       <c r="E38" s="66"/>
       <c r="F38" s="44"/>
       <c r="G38" s="44"/>
@@ -6264,6 +6217,102 @@
       <c r="T38" s="44"/>
       <c r="U38" s="33"/>
       <c r="V38" s="33"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="B39" s="29"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="2">
+        <v>800</v>
+      </c>
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="2">
+        <v>801</v>
+      </c>
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="2">
+        <v>802</v>
+      </c>
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="2">
+        <v>753</v>
+      </c>
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="2"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="E50" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">

</xml_diff>